<commit_message>
Add audited finance decision cases and correct valuation and calibration downloads
</commit_message>
<xml_diff>
--- a/projects/jbht-valuation/Quincy_Jones_JBHT_Three_Statement_DCF.xlsx
+++ b/projects/jbht-valuation/Quincy_Jones_JBHT_Three_Statement_DCF.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment Summary" sheetId="1" r:id="R9446532dad884e8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R7acbb38863ee46a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="3" r:id="R63a98b5d88fc41d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="4" r:id="R20ac843a03a042f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="5" r:id="Rdb23f343b70e40eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" r:id="R66cd8e9e96d544ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="7" r:id="R659b0fee5c2e42f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEC Actuals" sheetId="8" r:id="R40b3a7e94d464e37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R4174198088e24d06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Rb9f99cccc23a4e15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment Summary" sheetId="1" r:id="R911494090ed54ace"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R151071bc44044e6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="3" r:id="R3af654b956844eea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="4" r:id="R5cff96593d5c4922"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="5" r:id="Rfd76afba955c4b4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" r:id="R1438a5d6397d4349"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="7" r:id="R86f20ce547fe41f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEC Actuals" sheetId="8" r:id="R6201cb99f22942d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="Rf7413e5ac42f4a5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Ra85d67420abf4420"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -872,7 +872,7 @@
     </x:row>
     <x:row r="20" ht="26" customHeight="1">
       <x:c r="A20" s="79" t="str">
-        <x:v>Project application: Five years of SEC-reported financials, an integrated forecast, discounted cash flow, WACC / terminal-growth sensitivity, and trading comps. Applies methods from the CFI Valuation Modeling certificate.</x:v>
+        <x:v>Public-filings model with scenario valuation. Completed CFI valuation coursework informed the methods. Market data is a dated snapshot.</x:v>
       </x:c>
       <x:c r="B20" s="79"/>
       <x:c r="C20" s="79"/>
@@ -1678,7 +1678,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="8" t="str">
-        <x:v>Diluted shares implied by market cap / price (mm)</x:v>
+        <x:v>Market-implied shares (mm)</x:v>
       </x:c>
       <x:c r="B20" s="34" t="n">
         <x:v>94.944</x:v>
@@ -1755,90 +1755,90 @@
       <x:c r="J24" s="8"/>
       <x:c r="K24" s="8"/>
     </x:row>
-    <x:row r="25" ht="30" customHeight="1">
+    <x:row r="25" ht="44" customHeight="1">
       <x:c r="A25" s="39" t="str">
         <x:v>Net working capital</x:v>
       </x:c>
       <x:c r="B25" s="40" t="str">
         <x:v>Accounts receivable less accounts payable. Forecast cash flow reflects changes in these balances.</x:v>
       </x:c>
-      <x:c r="C25" s="41"/>
-      <x:c r="D25" s="41"/>
-      <x:c r="E25" s="41"/>
-      <x:c r="F25" s="41"/>
-      <x:c r="G25" s="41"/>
-      <x:c r="H25" s="41"/>
-      <x:c r="I25" s="41"/>
-      <x:c r="J25" s="41"/>
-      <x:c r="K25" s="41"/>
-    </x:row>
-    <x:row r="26" ht="30" customHeight="1">
+      <x:c r="C25" s="40"/>
+      <x:c r="D25" s="40"/>
+      <x:c r="E25" s="40"/>
+      <x:c r="F25" s="40"/>
+      <x:c r="G25" s="40"/>
+      <x:c r="H25" s="40"/>
+      <x:c r="I25" s="40"/>
+      <x:c r="J25" s="40"/>
+      <x:c r="K25" s="40"/>
+    </x:row>
+    <x:row r="26" ht="44" customHeight="1">
       <x:c r="A26" s="39" t="str">
         <x:v>Other assets and liabilities</x:v>
       </x:c>
       <x:c r="B26" s="40" t="str">
         <x:v>Held flat at FY2025 balances in the forecast.</x:v>
       </x:c>
-      <x:c r="C26" s="41"/>
-      <x:c r="D26" s="41"/>
-      <x:c r="E26" s="41"/>
-      <x:c r="F26" s="41"/>
-      <x:c r="G26" s="41"/>
-      <x:c r="H26" s="41"/>
-      <x:c r="I26" s="41"/>
-      <x:c r="J26" s="41"/>
-      <x:c r="K26" s="41"/>
-    </x:row>
-    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="C26" s="40"/>
+      <x:c r="D26" s="40"/>
+      <x:c r="E26" s="40"/>
+      <x:c r="F26" s="40"/>
+      <x:c r="G26" s="40"/>
+      <x:c r="H26" s="40"/>
+      <x:c r="I26" s="40"/>
+      <x:c r="J26" s="40"/>
+      <x:c r="K26" s="40"/>
+    </x:row>
+    <x:row r="27" ht="44" customHeight="1">
       <x:c r="A27" s="39" t="str">
         <x:v>Debt</x:v>
       </x:c>
       <x:c r="B27" s="40" t="str">
         <x:v>Held flat at FY2025 debt; no new borrowing or principal repayment assumed.</x:v>
       </x:c>
-      <x:c r="C27" s="41"/>
-      <x:c r="D27" s="41"/>
-      <x:c r="E27" s="41"/>
-      <x:c r="F27" s="41"/>
-      <x:c r="G27" s="41"/>
-      <x:c r="H27" s="41"/>
-      <x:c r="I27" s="41"/>
-      <x:c r="J27" s="41"/>
-      <x:c r="K27" s="41"/>
-    </x:row>
-    <x:row r="28" ht="30" customHeight="1">
+      <x:c r="C27" s="40"/>
+      <x:c r="D27" s="40"/>
+      <x:c r="E27" s="40"/>
+      <x:c r="F27" s="40"/>
+      <x:c r="G27" s="40"/>
+      <x:c r="H27" s="40"/>
+      <x:c r="I27" s="40"/>
+      <x:c r="J27" s="40"/>
+      <x:c r="K27" s="40"/>
+    </x:row>
+    <x:row r="28" ht="44" customHeight="1">
       <x:c r="A28" s="39" t="str">
         <x:v>Cash flow</x:v>
       </x:c>
       <x:c r="B28" s="40" t="str">
         <x:v>Forecast operating cash flow equals net income + D&amp;A − change in AR less AP.</x:v>
       </x:c>
-      <x:c r="C28" s="41"/>
-      <x:c r="D28" s="41"/>
-      <x:c r="E28" s="41"/>
-      <x:c r="F28" s="41"/>
-      <x:c r="G28" s="41"/>
-      <x:c r="H28" s="41"/>
-      <x:c r="I28" s="41"/>
-      <x:c r="J28" s="41"/>
-      <x:c r="K28" s="41"/>
-    </x:row>
-    <x:row r="29" ht="30" customHeight="1">
+      <x:c r="C28" s="40"/>
+      <x:c r="D28" s="40"/>
+      <x:c r="E28" s="40"/>
+      <x:c r="F28" s="40"/>
+      <x:c r="G28" s="40"/>
+      <x:c r="H28" s="40"/>
+      <x:c r="I28" s="40"/>
+      <x:c r="J28" s="40"/>
+      <x:c r="K28" s="40"/>
+    </x:row>
+    <x:row r="29" ht="44" customHeight="1">
       <x:c r="A29" s="39" t="str">
         <x:v>Shares</x:v>
       </x:c>
       <x:c r="B29" s="40" t="str">
-        <x:v>Share count is implied from market capitalization divided by share price and held flat.</x:v>
-      </x:c>
-      <x:c r="C29" s="41"/>
-      <x:c r="D29" s="41"/>
-      <x:c r="E29" s="41"/>
-      <x:c r="F29" s="41"/>
-      <x:c r="G29" s="41"/>
-      <x:c r="H29" s="41"/>
-      <x:c r="I29" s="41"/>
-      <x:c r="J29" s="41"/>
-      <x:c r="K29" s="41"/>
+        <x:v>Shares implied by the dated market cap / price snapshot; held flat. This is not weighted-average diluted EPS share count.</x:v>
+      </x:c>
+      <x:c r="C29" s="40"/>
+      <x:c r="D29" s="40"/>
+      <x:c r="E29" s="40"/>
+      <x:c r="F29" s="40"/>
+      <x:c r="G29" s="40"/>
+      <x:c r="H29" s="40"/>
+      <x:c r="I29" s="40"/>
+      <x:c r="J29" s="40"/>
+      <x:c r="K29" s="40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3719,7 +3719,7 @@
       </x:c>
       <x:c r="G7" s="8"/>
       <x:c r="H7" s="8" t="str">
-        <x:v>Enterprise value</x:v>
+        <x:v>Undiscounted terminal value</x:v>
       </x:c>
       <x:c r="I7" s="9" t="n">
         <x:f>F11*(1+Assumptions!$B$19)/(Assumptions!$B$18-Assumptions!$B$19)</x:f>
@@ -3851,7 +3851,7 @@
       </x:c>
       <x:c r="G11" s="8"/>
       <x:c r="H11" s="8" t="str">
-        <x:v>Diluted shares (mm)</x:v>
+        <x:v>Market-implied shares (mm)</x:v>
       </x:c>
       <x:c r="I11" s="53" t="n">
         <x:f>Assumptions!B20</x:f>
@@ -3971,8 +3971,13 @@
       <x:c r="E16" s="8"/>
       <x:c r="F16" s="8"/>
       <x:c r="G16" s="8"/>
-      <x:c r="H16" s="8"/>
-      <x:c r="I16" s="8"/>
+      <x:c r="H16" s="8" t="str">
+        <x:v>Enterprise value</x:v>
+      </x:c>
+      <x:c r="I16" s="53" t="n">
+        <x:f>SUM(I5:I6)</x:f>
+        <x:v>15687.2003130929</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8"/>

</xml_diff>